<commit_message>
Add geographic linkage review for local E5 disagreements
Extract sampled division, place-name, and Surrey council references from the 28 local E5 hard disagreements, and preserve the matching source sentences as review evidence. Add a separate Geographic Linkage worksheet so automated candidates remain clearly separated from the final human L1–L4 decisions.

Limit place matching to the 17 sampled divisions and their component place names to reduce false positives from generic ward names. Add tests for exact word-boundary matching and keep missing ward context explicit instead of inferring geographic eligibility.
</commit_message>
<xml_diff>
--- a/outputs/e5_disagreement_review_2026-07-24/E5_Hard_Disagreement_Review.xlsx
+++ b/outputs/e5_disagreement_review_2026-07-24/E5_Hard_Disagreement_Review.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R47857e80c9c14076"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="2" r:id="Rf985f5706d9f4338"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Article Text" sheetId="3" r:id="Rc17e9884c84d48a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="R1b311cd63d45467c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Lists" sheetId="5" r:id="R9b498978f7294345"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Independent Review" sheetId="6" r:id="Rf6679dd902da4c63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R1724179f3c324a08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="2" r:id="R9b4f9b3c4b94470d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Article Text" sheetId="3" r:id="R1560a68726274edd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" r:id="Rd2ab96616a1e4940"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Lists" sheetId="5" r:id="Rcf267e1f048143d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Independent Review" sheetId="6" r:id="R6f2b8d25e39647da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Geographic Linkage" sheetId="7" r:id="R7e3ed86d7674450d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,7 +22,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -67,8 +68,14 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1F1F1F"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="13">
+  <x:fills count="20">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -130,8 +137,43 @@
         <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCE6F1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F2F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDEBF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="16">
+  <x:borders count="17">
     <x:border/>
     <x:border>
       <x:right style="thin">
@@ -277,11 +319,25 @@
         <x:color rgb="FFD9D9D9"/>
       </x:top>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="92">
+  <x:cellXfs count="122">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -470,6 +526,68 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="11" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="15" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="15" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -758,6 +876,14 @@
         <x:v>Counts in Summary describe the development-set diagnosis only. They must not be reported as validation performance or used to authorise classification of the remaining corpus.</x:v>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="121" t="str">
+        <x:v>Geographic linkage</x:v>
+      </x:c>
+      <x:c r="B12" s="121" t="str">
+        <x:v>For the 28 local hard disagreements, use Geographic Linkage before final diagnosis. Automated candidates only locate possible evidence; confirm the sampled division/place and quote an exact sentence, or record why the linkage remains unresolved.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -9492,4 +9618,1273 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="38" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="55" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="22" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="24" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="55" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="25" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="42" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="22" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="14" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="10" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="24" customHeight="1">
+      <x:c r="A1" s="94" t="str">
+        <x:v>E5 local-arm geographic linkage review (28 hard disagreements)</x:v>
+      </x:c>
+      <x:c r="B1" s="94"/>
+      <x:c r="C1" s="94"/>
+      <x:c r="D1" s="94"/>
+      <x:c r="E1" s="94"/>
+      <x:c r="F1" s="94"/>
+      <x:c r="G1" s="94"/>
+      <x:c r="H1" s="94"/>
+      <x:c r="I1" s="94"/>
+      <x:c r="J1" s="94"/>
+      <x:c r="K1" s="94"/>
+      <x:c r="L1" s="94"/>
+      <x:c r="M1" s="94"/>
+      <x:c r="N1" s="94"/>
+      <x:c r="O1" s="94"/>
+      <x:c r="P1" s="94"/>
+      <x:c r="Q1" s="94"/>
+      <x:c r="R1" s="94"/>
+      <x:c r="S1" s="94"/>
+      <x:c r="T1" s="94"/>
+    </x:row>
+    <x:row r="2" ht="32" customHeight="1">
+      <x:c r="A2" s="97" t="str">
+        <x:v>Blue cells are deterministic search aids, not E5 decisions. Complete the yellow cells from the full article and record an exact supporting sentence before confirming L1-L4.</x:v>
+      </x:c>
+      <x:c r="B2" s="97"/>
+      <x:c r="C2" s="97"/>
+      <x:c r="D2" s="97"/>
+      <x:c r="E2" s="97"/>
+      <x:c r="F2" s="97"/>
+      <x:c r="G2" s="97"/>
+      <x:c r="H2" s="97"/>
+      <x:c r="I2" s="97"/>
+      <x:c r="J2" s="97"/>
+      <x:c r="K2" s="97"/>
+      <x:c r="L2" s="97"/>
+      <x:c r="M2" s="97"/>
+      <x:c r="N2" s="97"/>
+      <x:c r="O2" s="97"/>
+      <x:c r="P2" s="97"/>
+      <x:c r="Q2" s="97"/>
+      <x:c r="R2" s="97"/>
+      <x:c r="S2" s="97"/>
+      <x:c r="T2" s="97"/>
+    </x:row>
+    <x:row r="3" ht="32" customHeight="1">
+      <x:c r="A3" s="97" t="str">
+        <x:v>If the article names a place but the sampled division cannot be verified, choose unresolved_missing_context rather than inferring a ward.</x:v>
+      </x:c>
+      <x:c r="B3" s="97"/>
+      <x:c r="C3" s="97"/>
+      <x:c r="D3" s="97"/>
+      <x:c r="E3" s="97"/>
+      <x:c r="F3" s="97"/>
+      <x:c r="G3" s="97"/>
+      <x:c r="H3" s="97"/>
+      <x:c r="I3" s="97"/>
+      <x:c r="J3" s="97"/>
+      <x:c r="K3" s="97"/>
+      <x:c r="L3" s="97"/>
+      <x:c r="M3" s="97"/>
+      <x:c r="N3" s="97"/>
+      <x:c r="O3" s="97"/>
+      <x:c r="P3" s="97"/>
+      <x:c r="Q3" s="97"/>
+      <x:c r="R3" s="97"/>
+      <x:c r="S3" s="97"/>
+      <x:c r="T3" s="97"/>
+    </x:row>
+    <x:row r="5" ht="42" customHeight="1">
+      <x:c r="A5" s="111" t="str">
+        <x:v>review_index</x:v>
+      </x:c>
+      <x:c r="B5" s="111" t="str">
+        <x:v>article_id</x:v>
+      </x:c>
+      <x:c r="C5" s="111" t="str">
+        <x:v>headline</x:v>
+      </x:c>
+      <x:c r="D5" s="111" t="str">
+        <x:v>human_decision</x:v>
+      </x:c>
+      <x:c r="E5" s="111" t="str">
+        <x:v>llm_decision</x:v>
+      </x:c>
+      <x:c r="F5" s="111" t="str">
+        <x:v>ward_context_missing</x:v>
+      </x:c>
+      <x:c r="G5" s="111" t="str">
+        <x:v>exact_sample_division_candidates</x:v>
+      </x:c>
+      <x:c r="H5" s="111" t="str">
+        <x:v>sample_place_candidates</x:v>
+      </x:c>
+      <x:c r="I5" s="111" t="str">
+        <x:v>surrey_authority_signals</x:v>
+      </x:c>
+      <x:c r="J5" s="111" t="str">
+        <x:v>automated_evidence_sentences</x:v>
+      </x:c>
+      <x:c r="K5" s="111" t="str">
+        <x:v>linkage_review_status</x:v>
+      </x:c>
+      <x:c r="L5" s="111" t="str">
+        <x:v>confirmed_link_type</x:v>
+      </x:c>
+      <x:c r="M5" s="111" t="str">
+        <x:v>confirmed_linked_place</x:v>
+      </x:c>
+      <x:c r="N5" s="111" t="str">
+        <x:v>confirmed_sampled_division</x:v>
+      </x:c>
+      <x:c r="O5" s="111" t="str">
+        <x:v>confirmed_geographic_evidence</x:v>
+      </x:c>
+      <x:c r="P5" s="111" t="str">
+        <x:v>linkage_decision</x:v>
+      </x:c>
+      <x:c r="Q5" s="111" t="str">
+        <x:v>reviewer_notes</x:v>
+      </x:c>
+      <x:c r="R5" s="111" t="str">
+        <x:v>reviewer_id</x:v>
+      </x:c>
+      <x:c r="S5" s="111" t="str">
+        <x:v>reviewed_at</x:v>
+      </x:c>
+      <x:c r="T5" s="111" t="str">
+        <x:v>qc_flag</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="116" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B6" s="116" t="str">
+        <x:v>NEWS-bbc_surrey-26a6658188d3</x:v>
+      </x:c>
+      <x:c r="C6" s="116" t="str">
+        <x:v>Meningitis kills Surrey University student</x:v>
+      </x:c>
+      <x:c r="D6" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="E6" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="F6" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G6" s="117" t="str"/>
+      <x:c r="H6" s="117" t="str"/>
+      <x:c r="I6" s="117" t="str"/>
+      <x:c r="J6" s="117" t="str"/>
+      <x:c r="K6" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L6" s="118" t="str"/>
+      <x:c r="M6" s="118" t="str"/>
+      <x:c r="N6" s="118" t="str"/>
+      <x:c r="O6" s="118" t="str"/>
+      <x:c r="P6" s="118" t="str"/>
+      <x:c r="Q6" s="118" t="str"/>
+      <x:c r="R6" s="118" t="str"/>
+      <x:c r="S6" s="118" t="str"/>
+      <x:c r="T6" s="119" t="str">
+        <x:f>IF(K6&lt;&gt;"complete","",IF(OR(L6="",P6="",O6="",R6="",S6=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="116" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B7" s="116" t="str">
+        <x:v>NEWS-guardian_api-07bc83a03221</x:v>
+      </x:c>
+      <x:c r="C7" s="116" t="str">
+        <x:v>Starmer tells Labour MPs he is ‘not prepared to walk away’ after call for him to resign – as it happened </x:v>
+      </x:c>
+      <x:c r="D7" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="E7" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="F7" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G7" s="117" t="str"/>
+      <x:c r="H7" s="117" t="str"/>
+      <x:c r="I7" s="117" t="str"/>
+      <x:c r="J7" s="117" t="str"/>
+      <x:c r="K7" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L7" s="118" t="str"/>
+      <x:c r="M7" s="118" t="str"/>
+      <x:c r="N7" s="118" t="str"/>
+      <x:c r="O7" s="118" t="str"/>
+      <x:c r="P7" s="118" t="str"/>
+      <x:c r="Q7" s="118" t="str"/>
+      <x:c r="R7" s="118" t="str"/>
+      <x:c r="S7" s="118" t="str"/>
+      <x:c r="T7" s="119" t="str">
+        <x:f>IF(K7&lt;&gt;"complete","",IF(OR(L7="",P7="",O7="",R7="",S7=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="116" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B8" s="116" t="str">
+        <x:v>NEWS-guardian_api-0a2b7642ed1f</x:v>
+      </x:c>
+      <x:c r="C8" s="116" t="str">
+        <x:v>Could Lib Dems become the biggest party in English local government?</x:v>
+      </x:c>
+      <x:c r="D8" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="E8" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="F8" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G8" s="117" t="str"/>
+      <x:c r="H8" s="117" t="str"/>
+      <x:c r="I8" s="117" t="str"/>
+      <x:c r="J8" s="117" t="str"/>
+      <x:c r="K8" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L8" s="118" t="str"/>
+      <x:c r="M8" s="118" t="str"/>
+      <x:c r="N8" s="118" t="str"/>
+      <x:c r="O8" s="118" t="str"/>
+      <x:c r="P8" s="118" t="str"/>
+      <x:c r="Q8" s="118" t="str"/>
+      <x:c r="R8" s="118" t="str"/>
+      <x:c r="S8" s="118" t="str"/>
+      <x:c r="T8" s="119" t="str">
+        <x:f>IF(K8&lt;&gt;"complete","",IF(OR(L8="",P8="",O8="",R8="",S8=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="116" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B9" s="116" t="str">
+        <x:v>NEWS-guardian_api-0a8a98eec2fa</x:v>
+      </x:c>
+      <x:c r="C9" s="116" t="str">
+        <x:v>Funding gap of £643m puts  special needs teaching at risk</x:v>
+      </x:c>
+      <x:c r="D9" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="E9" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="F9" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G9" s="117" t="str"/>
+      <x:c r="H9" s="117" t="str"/>
+      <x:c r="I9" s="117" t="str">
+        <x:v>Surrey council</x:v>
+      </x:c>
+      <x:c r="J9" s="117" t="str">
+        <x:v>Surrey council cabinet member Julie Iles said: “We are proposing changes that provide the right level of support, and help young people to gain independence where possible and transition to adulthood successfully.</x:v>
+      </x:c>
+      <x:c r="K9" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L9" s="118" t="str"/>
+      <x:c r="M9" s="118" t="str"/>
+      <x:c r="N9" s="118" t="str"/>
+      <x:c r="O9" s="118" t="str"/>
+      <x:c r="P9" s="118" t="str"/>
+      <x:c r="Q9" s="118" t="str"/>
+      <x:c r="R9" s="118" t="str"/>
+      <x:c r="S9" s="118" t="str"/>
+      <x:c r="T9" s="119" t="str">
+        <x:f>IF(K9&lt;&gt;"complete","",IF(OR(L9="",P9="",O9="",R9="",S9=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="116" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B10" s="116" t="str">
+        <x:v>NEWS-guardian_api-0e7b3e16141a</x:v>
+      </x:c>
+      <x:c r="C10" s="116" t="str">
+        <x:v>UK politics: Government abandons plans to delay 30 local council elections in May – as it happened</x:v>
+      </x:c>
+      <x:c r="D10" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="E10" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="F10" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G10" s="117" t="str"/>
+      <x:c r="H10" s="117" t="str"/>
+      <x:c r="I10" s="117" t="str"/>
+      <x:c r="J10" s="117" t="str"/>
+      <x:c r="K10" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L10" s="118" t="str"/>
+      <x:c r="M10" s="118" t="str"/>
+      <x:c r="N10" s="118" t="str"/>
+      <x:c r="O10" s="118" t="str"/>
+      <x:c r="P10" s="118" t="str"/>
+      <x:c r="Q10" s="118" t="str"/>
+      <x:c r="R10" s="118" t="str"/>
+      <x:c r="S10" s="118" t="str"/>
+      <x:c r="T10" s="119" t="str">
+        <x:f>IF(K10&lt;&gt;"complete","",IF(OR(L10="",P10="",O10="",R10="",S10=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="116" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B11" s="116" t="str">
+        <x:v>NEWS-guardian_api-1593f58b94d2</x:v>
+      </x:c>
+      <x:c r="C11" s="116" t="str">
+        <x:v>Millwall stadium controversy intensifies as false funding claims revealed</x:v>
+      </x:c>
+      <x:c r="D11" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="E11" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="F11" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G11" s="117" t="str"/>
+      <x:c r="H11" s="117" t="str"/>
+      <x:c r="I11" s="117" t="str"/>
+      <x:c r="J11" s="117" t="str"/>
+      <x:c r="K11" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L11" s="118" t="str"/>
+      <x:c r="M11" s="118" t="str"/>
+      <x:c r="N11" s="118" t="str"/>
+      <x:c r="O11" s="118" t="str"/>
+      <x:c r="P11" s="118" t="str"/>
+      <x:c r="Q11" s="118" t="str"/>
+      <x:c r="R11" s="118" t="str"/>
+      <x:c r="S11" s="118" t="str"/>
+      <x:c r="T11" s="119" t="str">
+        <x:f>IF(K11&lt;&gt;"complete","",IF(OR(L11="",P11="",O11="",R11="",S11=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="116" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B12" s="116" t="str">
+        <x:v>NEWS-guardian_api-165b44f90fe0</x:v>
+      </x:c>
+      <x:c r="C12" s="116" t="str">
+        <x:v>The Guardian view on the last PMQs: now the unnecessary election | Editorial</x:v>
+      </x:c>
+      <x:c r="D12" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="E12" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="F12" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G12" s="117" t="str"/>
+      <x:c r="H12" s="117" t="str"/>
+      <x:c r="I12" s="117" t="str">
+        <x:v>Surrey council</x:v>
+      </x:c>
+      <x:c r="J12" s="117" t="str">
+        <x:v>Mr Corbyn did it in February when he read out leaked text exchanges between the leader of Surrey council and officials in the Department for Communities and Local Government, exposing a sweetheart deal over spending to avert a local referendum.</x:v>
+      </x:c>
+      <x:c r="K12" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L12" s="118" t="str"/>
+      <x:c r="M12" s="118" t="str"/>
+      <x:c r="N12" s="118" t="str"/>
+      <x:c r="O12" s="118" t="str"/>
+      <x:c r="P12" s="118" t="str"/>
+      <x:c r="Q12" s="118" t="str"/>
+      <x:c r="R12" s="118" t="str"/>
+      <x:c r="S12" s="118" t="str"/>
+      <x:c r="T12" s="119" t="str">
+        <x:f>IF(K12&lt;&gt;"complete","",IF(OR(L12="",P12="",O12="",R12="",S12=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="116" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B13" s="116" t="str">
+        <x:v>NEWS-guardian_api-299f68788499</x:v>
+      </x:c>
+      <x:c r="C13" s="116" t="str">
+        <x:v>Norovirus: people with winter vomiting bug urged to stay at home</x:v>
+      </x:c>
+      <x:c r="D13" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="E13" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="F13" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G13" s="117" t="str"/>
+      <x:c r="H13" s="117" t="str">
+        <x:v>Redhill</x:v>
+      </x:c>
+      <x:c r="I13" s="117" t="str"/>
+      <x:c r="J13" s="117" t="str">
+        <x:v>In the south of England East Surrey hospital in Redhill stopped visits to 10 of its wards on Tuesday, a decision which had not been taken lightly, Surrey and Sussex Healthcare NHS trust said.</x:v>
+      </x:c>
+      <x:c r="K13" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L13" s="118" t="str"/>
+      <x:c r="M13" s="118" t="str"/>
+      <x:c r="N13" s="118" t="str"/>
+      <x:c r="O13" s="118" t="str"/>
+      <x:c r="P13" s="118" t="str"/>
+      <x:c r="Q13" s="118" t="str"/>
+      <x:c r="R13" s="118" t="str"/>
+      <x:c r="S13" s="118" t="str"/>
+      <x:c r="T13" s="119" t="str">
+        <x:f>IF(K13&lt;&gt;"complete","",IF(OR(L13="",P13="",O13="",R13="",S13=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="116" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B14" s="116" t="str">
+        <x:v>NEWS-guardian_api-3a9be3f68624</x:v>
+      </x:c>
+      <x:c r="C14" s="116" t="str">
+        <x:v>‘I can’t sell mum’s retirement flat – and the charges are mounting up’</x:v>
+      </x:c>
+      <x:c r="D14" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="E14" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="F14" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G14" s="117" t="str"/>
+      <x:c r="H14" s="117" t="str"/>
+      <x:c r="I14" s="117" t="str"/>
+      <x:c r="J14" s="117" t="str"/>
+      <x:c r="K14" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L14" s="118" t="str"/>
+      <x:c r="M14" s="118" t="str"/>
+      <x:c r="N14" s="118" t="str"/>
+      <x:c r="O14" s="118" t="str"/>
+      <x:c r="P14" s="118" t="str"/>
+      <x:c r="Q14" s="118" t="str"/>
+      <x:c r="R14" s="118" t="str"/>
+      <x:c r="S14" s="118" t="str"/>
+      <x:c r="T14" s="119" t="str">
+        <x:f>IF(K14&lt;&gt;"complete","",IF(OR(L14="",P14="",O14="",R14="",S14=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="116" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B15" s="116" t="str">
+        <x:v>NEWS-guardian_api-4b66c98ae734</x:v>
+      </x:c>
+      <x:c r="C15" s="116" t="str">
+        <x:v>‘We’ve seen it decimate areas’: Somerset town’s traders oppose parking charges</x:v>
+      </x:c>
+      <x:c r="D15" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="E15" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="F15" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G15" s="117" t="str"/>
+      <x:c r="H15" s="117" t="str"/>
+      <x:c r="I15" s="117" t="str"/>
+      <x:c r="J15" s="117" t="str"/>
+      <x:c r="K15" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L15" s="118" t="str"/>
+      <x:c r="M15" s="118" t="str"/>
+      <x:c r="N15" s="118" t="str"/>
+      <x:c r="O15" s="118" t="str"/>
+      <x:c r="P15" s="118" t="str"/>
+      <x:c r="Q15" s="118" t="str"/>
+      <x:c r="R15" s="118" t="str"/>
+      <x:c r="S15" s="118" t="str"/>
+      <x:c r="T15" s="119" t="str">
+        <x:f>IF(K15&lt;&gt;"complete","",IF(OR(L15="",P15="",O15="",R15="",S15=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="116" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B16" s="116" t="str">
+        <x:v>NEWS-guardian_api-649bfee8381e</x:v>
+      </x:c>
+      <x:c r="C16" s="116" t="str">
+        <x:v>No 10 to delay four England mayoral elections amid accusations of ‘cancelling democracy’</x:v>
+      </x:c>
+      <x:c r="D16" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="E16" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="F16" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G16" s="117" t="str"/>
+      <x:c r="H16" s="117" t="str"/>
+      <x:c r="I16" s="117" t="str"/>
+      <x:c r="J16" s="117" t="str"/>
+      <x:c r="K16" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L16" s="118" t="str"/>
+      <x:c r="M16" s="118" t="str"/>
+      <x:c r="N16" s="118" t="str"/>
+      <x:c r="O16" s="118" t="str"/>
+      <x:c r="P16" s="118" t="str"/>
+      <x:c r="Q16" s="118" t="str"/>
+      <x:c r="R16" s="118" t="str"/>
+      <x:c r="S16" s="118" t="str"/>
+      <x:c r="T16" s="119" t="str">
+        <x:f>IF(K16&lt;&gt;"complete","",IF(OR(L16="",P16="",O16="",R16="",S16=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="116" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B17" s="116" t="str">
+        <x:v>NEWS-guardian_api-64ea38ced8bd</x:v>
+      </x:c>
+      <x:c r="C17" s="116" t="str">
+        <x:v>'After assembly, I cried': Surrey school grapples with race issues</x:v>
+      </x:c>
+      <x:c r="D17" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="E17" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="F17" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G17" s="117" t="str"/>
+      <x:c r="H17" s="117" t="str"/>
+      <x:c r="I17" s="117" t="str"/>
+      <x:c r="J17" s="117" t="str"/>
+      <x:c r="K17" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L17" s="118" t="str"/>
+      <x:c r="M17" s="118" t="str"/>
+      <x:c r="N17" s="118" t="str"/>
+      <x:c r="O17" s="118" t="str"/>
+      <x:c r="P17" s="118" t="str"/>
+      <x:c r="Q17" s="118" t="str"/>
+      <x:c r="R17" s="118" t="str"/>
+      <x:c r="S17" s="118" t="str"/>
+      <x:c r="T17" s="119" t="str">
+        <x:f>IF(K17&lt;&gt;"complete","",IF(OR(L17="",P17="",O17="",R17="",S17=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="116" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B18" s="116" t="str">
+        <x:v>NEWS-guardian_api-6549611cf8a4</x:v>
+      </x:c>
+      <x:c r="C18" s="116" t="str">
+        <x:v>‘The government must unlock the money. Because the care crisis is now’   | Hélène Mulholland</x:v>
+      </x:c>
+      <x:c r="D18" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="E18" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="F18" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G18" s="117" t="str"/>
+      <x:c r="H18" s="117" t="str"/>
+      <x:c r="I18" s="117" t="str"/>
+      <x:c r="J18" s="117" t="str"/>
+      <x:c r="K18" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L18" s="118" t="str"/>
+      <x:c r="M18" s="118" t="str"/>
+      <x:c r="N18" s="118" t="str"/>
+      <x:c r="O18" s="118" t="str"/>
+      <x:c r="P18" s="118" t="str"/>
+      <x:c r="Q18" s="118" t="str"/>
+      <x:c r="R18" s="118" t="str"/>
+      <x:c r="S18" s="118" t="str"/>
+      <x:c r="T18" s="119" t="str">
+        <x:f>IF(K18&lt;&gt;"complete","",IF(OR(L18="",P18="",O18="",R18="",S18=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="116" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B19" s="116" t="str">
+        <x:v>NEWS-guardian_api-6d0b3b8aedc2</x:v>
+      </x:c>
+      <x:c r="C19" s="116" t="str">
+        <x:v>Millwall admit council scheme could force club to leave Lewisham</x:v>
+      </x:c>
+      <x:c r="D19" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="E19" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="F19" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G19" s="117" t="str"/>
+      <x:c r="H19" s="117" t="str"/>
+      <x:c r="I19" s="117" t="str"/>
+      <x:c r="J19" s="117" t="str"/>
+      <x:c r="K19" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L19" s="118" t="str"/>
+      <x:c r="M19" s="118" t="str"/>
+      <x:c r="N19" s="118" t="str"/>
+      <x:c r="O19" s="118" t="str"/>
+      <x:c r="P19" s="118" t="str"/>
+      <x:c r="Q19" s="118" t="str"/>
+      <x:c r="R19" s="118" t="str"/>
+      <x:c r="S19" s="118" t="str"/>
+      <x:c r="T19" s="119" t="str">
+        <x:f>IF(K19&lt;&gt;"complete","",IF(OR(L19="",P19="",O19="",R19="",S19=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="116" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B20" s="116" t="str">
+        <x:v>NEWS-guardian_api-6d2d7efbb858</x:v>
+      </x:c>
+      <x:c r="C20" s="116" t="str">
+        <x:v>Spirit of Margaret Thatcher invoked by Tory backers of gay marriage</x:v>
+      </x:c>
+      <x:c r="D20" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="E20" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="F20" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G20" s="117" t="str"/>
+      <x:c r="H20" s="117" t="str"/>
+      <x:c r="I20" s="117" t="str"/>
+      <x:c r="J20" s="117" t="str"/>
+      <x:c r="K20" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L20" s="118" t="str"/>
+      <x:c r="M20" s="118" t="str"/>
+      <x:c r="N20" s="118" t="str"/>
+      <x:c r="O20" s="118" t="str"/>
+      <x:c r="P20" s="118" t="str"/>
+      <x:c r="Q20" s="118" t="str"/>
+      <x:c r="R20" s="118" t="str"/>
+      <x:c r="S20" s="118" t="str"/>
+      <x:c r="T20" s="119" t="str">
+        <x:f>IF(K20&lt;&gt;"complete","",IF(OR(L20="",P20="",O20="",R20="",S20=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="116" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B21" s="116" t="str">
+        <x:v>NEWS-guardian_api-8c28af0f119c</x:v>
+      </x:c>
+      <x:c r="C21" s="116" t="str">
+        <x:v>Badenoch says teaching boys about misogyny shouldn’t be a priority because migrants more dangerous to women and girls – UK politics live</x:v>
+      </x:c>
+      <x:c r="D21" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="E21" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="F21" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G21" s="117" t="str"/>
+      <x:c r="H21" s="117" t="str"/>
+      <x:c r="I21" s="117" t="str"/>
+      <x:c r="J21" s="117" t="str"/>
+      <x:c r="K21" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L21" s="118" t="str"/>
+      <x:c r="M21" s="118" t="str"/>
+      <x:c r="N21" s="118" t="str"/>
+      <x:c r="O21" s="118" t="str"/>
+      <x:c r="P21" s="118" t="str"/>
+      <x:c r="Q21" s="118" t="str"/>
+      <x:c r="R21" s="118" t="str"/>
+      <x:c r="S21" s="118" t="str"/>
+      <x:c r="T21" s="119" t="str">
+        <x:f>IF(K21&lt;&gt;"complete","",IF(OR(L21="",P21="",O21="",R21="",S21=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="116" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B22" s="116" t="str">
+        <x:v>NEWS-guardian_api-8e547ee6efe6</x:v>
+      </x:c>
+      <x:c r="C22" s="116" t="str">
+        <x:v>UK politics: Farage insults female reporter as Braverman says Reform UK wants to scrap Equality Act – as it happened</x:v>
+      </x:c>
+      <x:c r="D22" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="E22" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="F22" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G22" s="117" t="str"/>
+      <x:c r="H22" s="117" t="str"/>
+      <x:c r="I22" s="117" t="str">
+        <x:v>Surrey councillor</x:v>
+      </x:c>
+      <x:c r="J22" s="117" t="str">
+        <x:v>On C4News tonight, Gary Gibbon tells the story - based on my biography - of how in 2004, while a Ukip MEP, Farage secretly met a senior Cons MP &amp;amp; a Surrey councillor, seeking their help to defect &amp;amp; get picked for a safe Tory seat.</x:v>
+      </x:c>
+      <x:c r="K22" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L22" s="118" t="str"/>
+      <x:c r="M22" s="118" t="str"/>
+      <x:c r="N22" s="118" t="str"/>
+      <x:c r="O22" s="118" t="str"/>
+      <x:c r="P22" s="118" t="str"/>
+      <x:c r="Q22" s="118" t="str"/>
+      <x:c r="R22" s="118" t="str"/>
+      <x:c r="S22" s="118" t="str"/>
+      <x:c r="T22" s="119" t="str">
+        <x:f>IF(K22&lt;&gt;"complete","",IF(OR(L22="",P22="",O22="",R22="",S22=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="116" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B23" s="116" t="str">
+        <x:v>NEWS-guardian_api-8f8e97810c4d</x:v>
+      </x:c>
+      <x:c r="C23" s="116" t="str">
+        <x:v>Covid rules out Boxing Day hunts and parades amid uncertain future</x:v>
+      </x:c>
+      <x:c r="D23" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="E23" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="F23" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G23" s="117" t="str"/>
+      <x:c r="H23" s="117" t="str"/>
+      <x:c r="I23" s="117" t="str"/>
+      <x:c r="J23" s="117" t="str"/>
+      <x:c r="K23" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L23" s="118" t="str"/>
+      <x:c r="M23" s="118" t="str"/>
+      <x:c r="N23" s="118" t="str"/>
+      <x:c r="O23" s="118" t="str"/>
+      <x:c r="P23" s="118" t="str"/>
+      <x:c r="Q23" s="118" t="str"/>
+      <x:c r="R23" s="118" t="str"/>
+      <x:c r="S23" s="118" t="str"/>
+      <x:c r="T23" s="119" t="str">
+        <x:f>IF(K23&lt;&gt;"complete","",IF(OR(L23="",P23="",O23="",R23="",S23=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="116" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B24" s="116" t="str">
+        <x:v>NEWS-guardian_api-9dea17fa1487</x:v>
+      </x:c>
+      <x:c r="C24" s="116" t="str">
+        <x:v>England's new Covid rules: what is allowed in tiers 1, 2 and 3?</x:v>
+      </x:c>
+      <x:c r="D24" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="E24" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="F24" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G24" s="117" t="str"/>
+      <x:c r="H24" s="117" t="str"/>
+      <x:c r="I24" s="117" t="str"/>
+      <x:c r="J24" s="117" t="str"/>
+      <x:c r="K24" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L24" s="118" t="str"/>
+      <x:c r="M24" s="118" t="str"/>
+      <x:c r="N24" s="118" t="str"/>
+      <x:c r="O24" s="118" t="str"/>
+      <x:c r="P24" s="118" t="str"/>
+      <x:c r="Q24" s="118" t="str"/>
+      <x:c r="R24" s="118" t="str"/>
+      <x:c r="S24" s="118" t="str"/>
+      <x:c r="T24" s="119" t="str">
+        <x:f>IF(K24&lt;&gt;"complete","",IF(OR(L24="",P24="",O24="",R24="",S24=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="116" t="n">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B25" s="116" t="str">
+        <x:v>NEWS-guardian_api-ab4a777c619a</x:v>
+      </x:c>
+      <x:c r="C25" s="116" t="str">
+        <x:v>ID cards and wider issues of voter engagement | Letters</x:v>
+      </x:c>
+      <x:c r="D25" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="E25" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="F25" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G25" s="117" t="str"/>
+      <x:c r="H25" s="117" t="str"/>
+      <x:c r="I25" s="117" t="str"/>
+      <x:c r="J25" s="117" t="str"/>
+      <x:c r="K25" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L25" s="118" t="str"/>
+      <x:c r="M25" s="118" t="str"/>
+      <x:c r="N25" s="118" t="str"/>
+      <x:c r="O25" s="118" t="str"/>
+      <x:c r="P25" s="118" t="str"/>
+      <x:c r="Q25" s="118" t="str"/>
+      <x:c r="R25" s="118" t="str"/>
+      <x:c r="S25" s="118" t="str"/>
+      <x:c r="T25" s="119" t="str">
+        <x:f>IF(K25&lt;&gt;"complete","",IF(OR(L25="",P25="",O25="",R25="",S25=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="116" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B26" s="116" t="str">
+        <x:v>NEWS-guardian_api-b48d01a86b76</x:v>
+      </x:c>
+      <x:c r="C26" s="116" t="str">
+        <x:v>Police to question Andrew’s former protection officers over his Epstein links</x:v>
+      </x:c>
+      <x:c r="D26" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="E26" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="F26" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G26" s="117" t="str"/>
+      <x:c r="H26" s="117" t="str"/>
+      <x:c r="I26" s="117" t="str"/>
+      <x:c r="J26" s="117" t="str"/>
+      <x:c r="K26" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L26" s="118" t="str"/>
+      <x:c r="M26" s="118" t="str"/>
+      <x:c r="N26" s="118" t="str"/>
+      <x:c r="O26" s="118" t="str"/>
+      <x:c r="P26" s="118" t="str"/>
+      <x:c r="Q26" s="118" t="str"/>
+      <x:c r="R26" s="118" t="str"/>
+      <x:c r="S26" s="118" t="str"/>
+      <x:c r="T26" s="119" t="str">
+        <x:f>IF(K26&lt;&gt;"complete","",IF(OR(L26="",P26="",O26="",R26="",S26=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="116" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="B27" s="116" t="str">
+        <x:v>NEWS-guardian_api-b9d210492f43</x:v>
+      </x:c>
+      <x:c r="C27" s="116" t="str">
+        <x:v>Explainer: what are the new Covid rules in the UK from Boxing Day?</x:v>
+      </x:c>
+      <x:c r="D27" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="E27" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="F27" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G27" s="117" t="str"/>
+      <x:c r="H27" s="117" t="str"/>
+      <x:c r="I27" s="117" t="str"/>
+      <x:c r="J27" s="117" t="str"/>
+      <x:c r="K27" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L27" s="118" t="str"/>
+      <x:c r="M27" s="118" t="str"/>
+      <x:c r="N27" s="118" t="str"/>
+      <x:c r="O27" s="118" t="str"/>
+      <x:c r="P27" s="118" t="str"/>
+      <x:c r="Q27" s="118" t="str"/>
+      <x:c r="R27" s="118" t="str"/>
+      <x:c r="S27" s="118" t="str"/>
+      <x:c r="T27" s="119" t="str">
+        <x:f>IF(K27&lt;&gt;"complete","",IF(OR(L27="",P27="",O27="",R27="",S27=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="116" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B28" s="116" t="str">
+        <x:v>NEWS-guardian_api-cc8e272342e5</x:v>
+      </x:c>
+      <x:c r="C28" s="116" t="str">
+        <x:v>Enver Solomon restores our faith in Britain | Letters</x:v>
+      </x:c>
+      <x:c r="D28" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="E28" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="F28" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G28" s="117" t="str"/>
+      <x:c r="H28" s="117" t="str"/>
+      <x:c r="I28" s="117" t="str"/>
+      <x:c r="J28" s="117" t="str"/>
+      <x:c r="K28" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L28" s="118" t="str"/>
+      <x:c r="M28" s="118" t="str"/>
+      <x:c r="N28" s="118" t="str"/>
+      <x:c r="O28" s="118" t="str"/>
+      <x:c r="P28" s="118" t="str"/>
+      <x:c r="Q28" s="118" t="str"/>
+      <x:c r="R28" s="118" t="str"/>
+      <x:c r="S28" s="118" t="str"/>
+      <x:c r="T28" s="119" t="str">
+        <x:f>IF(K28&lt;&gt;"complete","",IF(OR(L28="",P28="",O28="",R28="",S28=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="116" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="B29" s="116" t="str">
+        <x:v>NEWS-guardian_api-d12e8db585f0</x:v>
+      </x:c>
+      <x:c r="C29" s="116" t="str">
+        <x:v>Flawed council shake-up plans will not deliver savings | Letters</x:v>
+      </x:c>
+      <x:c r="D29" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="E29" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="F29" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G29" s="117" t="str"/>
+      <x:c r="H29" s="117" t="str">
+        <x:v>Guildford</x:v>
+      </x:c>
+      <x:c r="I29" s="117" t="str"/>
+      <x:c r="J29" s="117" t="str">
+        <x:v>Bernard Quoroll Guildford, Surrey • Why Labour is wasting energy on an unnecessary reform of local government is, as Polly Toynbee points out, puzzling.</x:v>
+      </x:c>
+      <x:c r="K29" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L29" s="118" t="str"/>
+      <x:c r="M29" s="118" t="str"/>
+      <x:c r="N29" s="118" t="str"/>
+      <x:c r="O29" s="118" t="str"/>
+      <x:c r="P29" s="118" t="str"/>
+      <x:c r="Q29" s="118" t="str"/>
+      <x:c r="R29" s="118" t="str"/>
+      <x:c r="S29" s="118" t="str"/>
+      <x:c r="T29" s="119" t="str">
+        <x:f>IF(K29&lt;&gt;"complete","",IF(OR(L29="",P29="",O29="",R29="",S29=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="116" t="n">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="B30" s="116" t="str">
+        <x:v>NEWS-guardian_api-de14fda465d9</x:v>
+      </x:c>
+      <x:c r="C30" s="116" t="str">
+        <x:v>I've been unfairly targeted, says academic at heart of National Trust 'woke' row</x:v>
+      </x:c>
+      <x:c r="D30" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="E30" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="F30" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G30" s="117" t="str"/>
+      <x:c r="H30" s="117" t="str"/>
+      <x:c r="I30" s="117" t="str"/>
+      <x:c r="J30" s="117" t="str"/>
+      <x:c r="K30" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L30" s="118" t="str"/>
+      <x:c r="M30" s="118" t="str"/>
+      <x:c r="N30" s="118" t="str"/>
+      <x:c r="O30" s="118" t="str"/>
+      <x:c r="P30" s="118" t="str"/>
+      <x:c r="Q30" s="118" t="str"/>
+      <x:c r="R30" s="118" t="str"/>
+      <x:c r="S30" s="118" t="str"/>
+      <x:c r="T30" s="119" t="str">
+        <x:f>IF(K30&lt;&gt;"complete","",IF(OR(L30="",P30="",O30="",R30="",S30=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="116" t="n">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="B31" s="116" t="str">
+        <x:v>NEWS-guardian_api-e9ed22adbdb1</x:v>
+      </x:c>
+      <x:c r="C31" s="116" t="str">
+        <x:v>A new year brings new battles for democracy and for Labour | Letters </x:v>
+      </x:c>
+      <x:c r="D31" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="E31" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="F31" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G31" s="117" t="str"/>
+      <x:c r="H31" s="117" t="str">
+        <x:v>Farnham</x:v>
+      </x:c>
+      <x:c r="I31" s="117" t="str"/>
+      <x:c r="J31" s="117" t="str">
+        <x:v>Tom Quinn Farnham, Surrey • Have an opinion on anything you’ve read in the Guardian today?</x:v>
+      </x:c>
+      <x:c r="K31" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L31" s="118" t="str"/>
+      <x:c r="M31" s="118" t="str"/>
+      <x:c r="N31" s="118" t="str"/>
+      <x:c r="O31" s="118" t="str"/>
+      <x:c r="P31" s="118" t="str"/>
+      <x:c r="Q31" s="118" t="str"/>
+      <x:c r="R31" s="118" t="str"/>
+      <x:c r="S31" s="118" t="str"/>
+      <x:c r="T31" s="119" t="str">
+        <x:f>IF(K31&lt;&gt;"complete","",IF(OR(L31="",P31="",O31="",R31="",S31=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="116" t="n">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B32" s="116" t="str">
+        <x:v>NEWS-guardian_api-f0e1fbfa261a</x:v>
+      </x:c>
+      <x:c r="C32" s="116" t="str">
+        <x:v>Today in healthcare: Tuesday 22 January</x:v>
+      </x:c>
+      <x:c r="D32" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="E32" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="F32" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G32" s="117" t="str"/>
+      <x:c r="H32" s="117" t="str"/>
+      <x:c r="I32" s="117" t="str"/>
+      <x:c r="J32" s="117" t="str"/>
+      <x:c r="K32" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L32" s="118" t="str"/>
+      <x:c r="M32" s="118" t="str"/>
+      <x:c r="N32" s="118" t="str"/>
+      <x:c r="O32" s="118" t="str"/>
+      <x:c r="P32" s="118" t="str"/>
+      <x:c r="Q32" s="118" t="str"/>
+      <x:c r="R32" s="118" t="str"/>
+      <x:c r="S32" s="118" t="str"/>
+      <x:c r="T32" s="119" t="str">
+        <x:f>IF(K32&lt;&gt;"complete","",IF(OR(L32="",P32="",O32="",R32="",S32=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="116" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="B33" s="116" t="str">
+        <x:v>NEWS-guardian_api-ffae95f17052</x:v>
+      </x:c>
+      <x:c r="C33" s="116" t="str">
+        <x:v>‘An abomination’: the Lancashire town kicking up a stink over reopened landfill</x:v>
+      </x:c>
+      <x:c r="D33" s="116" t="str">
+        <x:v>exclude</x:v>
+      </x:c>
+      <x:c r="E33" s="116" t="str">
+        <x:v>include</x:v>
+      </x:c>
+      <x:c r="F33" s="116" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G33" s="117" t="str"/>
+      <x:c r="H33" s="117" t="str"/>
+      <x:c r="I33" s="117" t="str"/>
+      <x:c r="J33" s="117" t="str"/>
+      <x:c r="K33" s="118" t="str">
+        <x:v>not_started</x:v>
+      </x:c>
+      <x:c r="L33" s="118" t="str"/>
+      <x:c r="M33" s="118" t="str"/>
+      <x:c r="N33" s="118" t="str"/>
+      <x:c r="O33" s="118" t="str"/>
+      <x:c r="P33" s="118" t="str"/>
+      <x:c r="Q33" s="118" t="str"/>
+      <x:c r="R33" s="118" t="str"/>
+      <x:c r="S33" s="118" t="str"/>
+      <x:c r="T33" s="119" t="str">
+        <x:f>IF(K33&lt;&gt;"complete","",IF(OR(L33="",P33="",O33="",R33="",S33=""),"CHECK","OK"))</x:f>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:T1"/>
+    <x:mergeCell ref="A2:T2"/>
+    <x:mergeCell ref="A3:T3"/>
+  </x:mergeCells>
+  <x:dataValidations count="3">
+    <x:dataValidation type="list" sqref="K6:K33">
+      <x:formula1>"not_started,in_progress,complete,needs_adjudication"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="L6:L33">
+      <x:formula1>"L1_place,L2_candidate,L3_council_issue,L4_county_wide,no_link"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="P6:P33">
+      <x:formula1>"confirmed,rejected_incidental,unresolved_missing_context,not_applicable"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>